<commit_message>
Adding lots of additional support for Discourse bot, minor bug fixes. See changelog.md
</commit_message>
<xml_diff>
--- a/sample_transactions.xlsx
+++ b/sample_transactions.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wojciech/Wojciech-Dev-Space/agenticportfolio/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wojciech/Wojciech-Dev-Space/athena-os-official/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E34FFD31-CBF1-9546-BBCF-A2A1D5D34381}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23EE699F-D369-AF49-A1A7-1C8DBBABB9A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2600" yWindow="2500" windowWidth="25820" windowHeight="14940" xr2:uid="{10D8B0BF-8D59-B248-B5C4-343822590B80}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
   <si>
     <t>SYMBOL</t>
   </si>
@@ -72,13 +72,19 @@
   </si>
   <si>
     <t>SELL</t>
+  </si>
+  <si>
+    <t>CASH_IN</t>
+  </si>
+  <si>
+    <t>n/a</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -88,6 +94,12 @@
     </font>
     <font>
       <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -114,9 +126,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -451,7 +465,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{438BC79E-4821-234F-88E1-B54FFF9A889B}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="23.83203125" bestFit="1" customWidth="1"/>
@@ -478,23 +492,23 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+    <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="3">
+        <v>45992</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2">
-        <v>100</v>
-      </c>
-      <c r="E2">
-        <v>2</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="E2" s="2">
+        <v>200</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -503,10 +517,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D3">
         <v>100</v>
@@ -515,6 +529,26 @@
         <v>2</v>
       </c>
       <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4">
+        <v>100</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>